<commit_message>
B&N step 9: alcances OK, registro entregable, reglas OK except back-check; plantilla/familias/alcances 1/2in sheathing family (R80e.16)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UQBQT8jCVU6KW8QmKhZS83
</commit_message>
<xml_diff>
--- a/cache_proyectos/barnes_noble/takeoff_work/etapas/8_excel/Barnes_Noble_ColoradoSprings_Takeoff_FINAL.xlsx
+++ b/cache_proyectos/barnes_noble/takeoff_work/etapas/8_excel/Barnes_Noble_ColoradoSprings_Takeoff_FINAL.xlsx
@@ -1258,13 +1258,13 @@
     <t xml:space="preserve">SF</t>
   </si>
   <si>
-    <t xml:space="preserve">piece</t>
+    <t xml:space="preserve">4x8 ft sheet</t>
   </si>
   <si>
     <t xml:space="preserve">familias_out.json '5/8" gyp board regular (walls + ceilings)' (R80.4: canon family the run did not write)</t>
   </si>
   <si>
-    <t xml:space="preserve">1/2" EXTERIOR gyp sheathing</t>
+    <t xml:space="preserve">1/2" EXTERIOR gypsum sheathing</t>
   </si>
   <si>
     <t xml:space="preserve">familias_out.json '1/2" EXTERIOR gyp sheathing' (R80.4: canon family the run did not write)</t>
@@ -1279,7 +1279,7 @@
     <t xml:space="preserve">familias_out.json 'metal trim (corner bead, casing, shadow molding)' (R80.4: canon family the run did not write)</t>
   </si>
   <si>
-    <t xml:space="preserve">Cement board (substrate under the FRP cove base band)</t>
+    <t xml:space="preserve">Cement board (tile / FRP substrate)</t>
   </si>
   <si>
     <t xml:space="preserve">familias_out.json 'cement board' (R80.4: canon family the run did not write)</t>
@@ -6714,23 +6714,23 @@
         <v>16562.77</v>
       </c>
       <c r="D20" s="0" t="n">
-        <f aca="false">Inputs!$B$5</f>
-        <v>0.15</v>
+        <f aca="false">Inputs!$B$6</f>
+        <v>0.06</v>
       </c>
       <c r="E20" s="0" t="n">
         <f aca="false">C20*D20</f>
-        <v>2484.4155</v>
+        <v>993.7662</v>
       </c>
       <c r="F20" s="0" t="n">
         <f aca="false">C20+E20</f>
-        <v>19047.1855</v>
+        <v>17556.5362</v>
       </c>
       <c r="G20" s="0" t="s">
         <v>410</v>
       </c>
       <c r="H20" s="0" t="n">
-        <f aca="false">ROUNDUP(F20,0)</f>
-        <v>19048</v>
+        <f aca="false">ROUNDUP(F20/32,0)</f>
+        <v>549</v>
       </c>
       <c r="I20" s="0" t="s">
         <v>411</v>
@@ -6741,29 +6741,29 @@
         <v>412</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>378</v>
+        <v>409</v>
       </c>
       <c r="C21" s="0" t="n">
         <v>2469.22</v>
       </c>
       <c r="D21" s="0" t="n">
-        <f aca="false">Inputs!$B$5</f>
-        <v>0.15</v>
+        <f aca="false">Inputs!$B$6</f>
+        <v>0.06</v>
       </c>
       <c r="E21" s="0" t="n">
         <f aca="false">C21*D21</f>
-        <v>370.383</v>
+        <v>148.1532</v>
       </c>
       <c r="F21" s="0" t="n">
         <f aca="false">C21+E21</f>
-        <v>2839.603</v>
+        <v>2617.3732</v>
       </c>
       <c r="G21" s="0" t="s">
         <v>410</v>
       </c>
       <c r="H21" s="0" t="n">
-        <f aca="false">ROUNDUP(F21,0)</f>
-        <v>2840</v>
+        <f aca="false">ROUNDUP(F21/32,0)</f>
+        <v>82</v>
       </c>
       <c r="I21" s="0" t="s">
         <v>413</v>
@@ -6813,23 +6813,23 @@
         <v>851.4</v>
       </c>
       <c r="D23" s="0" t="n">
-        <f aca="false">Inputs!$B$5</f>
-        <v>0.15</v>
+        <f aca="false">Inputs!$B$6</f>
+        <v>0.06</v>
       </c>
       <c r="E23" s="0" t="n">
         <f aca="false">C23*D23</f>
-        <v>127.71</v>
+        <v>51.084</v>
       </c>
       <c r="F23" s="0" t="n">
         <f aca="false">C23+E23</f>
-        <v>979.11</v>
+        <v>902.484</v>
       </c>
       <c r="G23" s="0" t="s">
         <v>410</v>
       </c>
       <c r="H23" s="0" t="n">
-        <f aca="false">ROUNDUP(F23,0)</f>
-        <v>980</v>
+        <f aca="false">ROUNDUP(F23/32,0)</f>
+        <v>29</v>
       </c>
       <c r="I23" s="0" t="s">
         <v>418</v>

</xml_diff>

<commit_message>
B&N step 9 gates passed: back-check (PASS WITH COMMENTS, finding 2 fixed), reglas OK, alcances OK, registro entregable, etapas PASA, BITACORA OK (R80e.17)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UQBQT8jCVU6KW8QmKhZS83
</commit_message>
<xml_diff>
--- a/cache_proyectos/barnes_noble/takeoff_work/etapas/8_excel/Barnes_Noble_ColoradoSprings_Takeoff_FINAL.xlsx
+++ b/cache_proyectos/barnes_noble/takeoff_work/etapas/8_excel/Barnes_Noble_ColoradoSprings_Takeoff_FINAL.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1060" uniqueCount="693">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1060" uniqueCount="692">
   <si>
     <t xml:space="preserve">Barnes &amp; Noble - Colorado Springs, CO (3173 Cinema Point)   |   METAL FRAMING &amp; DRYWALL TAKEOFF</t>
   </si>
@@ -1258,7 +1258,7 @@
     <t xml:space="preserve">SF</t>
   </si>
   <si>
-    <t xml:space="preserve">4x8 ft sheet</t>
+    <t xml:space="preserve">4x12 ft sheet (Inputs)</t>
   </si>
   <si>
     <t xml:space="preserve">familias_out.json '5/8" gyp board regular (walls + ceilings)' (R80.4: canon family the run did not write)</t>
@@ -1292,9 +1292,6 @@
   </si>
   <si>
     <t xml:space="preserve">FRT plywood substrate (5/8 in.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4x12 ft sheet (Inputs)</t>
   </si>
   <si>
     <t xml:space="preserve">familias_out.json FRT plywood by material; canon rows</t>
@@ -6729,8 +6726,8 @@
         <v>410</v>
       </c>
       <c r="H20" s="0" t="n">
-        <f aca="false">ROUNDUP(F20/32,0)</f>
-        <v>549</v>
+        <f aca="false">ROUNDUP(F20/Inputs!$B$9,0)</f>
+        <v>366</v>
       </c>
       <c r="I20" s="0" t="s">
         <v>411</v>
@@ -6762,8 +6759,8 @@
         <v>410</v>
       </c>
       <c r="H21" s="0" t="n">
-        <f aca="false">ROUNDUP(F21/32,0)</f>
-        <v>82</v>
+        <f aca="false">ROUNDUP(F21/Inputs!$B$9,0)</f>
+        <v>55</v>
       </c>
       <c r="I21" s="0" t="s">
         <v>413</v>
@@ -6828,8 +6825,8 @@
         <v>410</v>
       </c>
       <c r="H23" s="0" t="n">
-        <f aca="false">ROUNDUP(F23/32,0)</f>
-        <v>29</v>
+        <f aca="false">ROUNDUP(F23/Inputs!$B$9,0)</f>
+        <v>19</v>
       </c>
       <c r="I23" s="0" t="s">
         <v>418</v>
@@ -6891,19 +6888,19 @@
         <v>2680.1252</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>422</v>
+        <v>410</v>
       </c>
       <c r="H25" s="0" t="n">
         <f aca="false">ROUNDUP(F25/Inputs!$B$9,0)</f>
         <v>56</v>
       </c>
       <c r="I25" s="0" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B26" s="0" t="s">
         <v>409</v>
@@ -6924,22 +6921,22 @@
         <v>67.2888</v>
       </c>
       <c r="G26" s="0" t="s">
-        <v>422</v>
+        <v>410</v>
       </c>
       <c r="H26" s="0" t="n">
         <f aca="false">ROUNDUP(F26/Inputs!$B$9,0)</f>
         <v>2</v>
       </c>
       <c r="I26" s="0" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
+        <v>424</v>
+      </c>
+      <c r="B27" s="0" t="s">
         <v>425</v>
-      </c>
-      <c r="B27" s="0" t="s">
-        <v>426</v>
       </c>
       <c r="C27" s="0" t="n">
         <v>103</v>
@@ -6960,12 +6957,12 @@
         <v>103</v>
       </c>
       <c r="I27" s="0" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B28" s="0" t="s">
         <v>378</v>
@@ -6993,15 +6990,15 @@
         <v>3</v>
       </c>
       <c r="I28" s="0" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C29" s="0" t="n">
         <v>0</v>
@@ -7018,19 +7015,19 @@
         <v>0</v>
       </c>
       <c r="G29" s="0" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="H29" s="0" t="n">
         <f aca="false">ROUNDUP(F29,0)</f>
         <v>0</v>
       </c>
       <c r="I29" s="0" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B30" s="0" t="s">
         <v>378</v>
@@ -7058,12 +7055,12 @@
         <v>0</v>
       </c>
       <c r="I30" s="0" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B31" s="0" t="s">
         <v>378</v>
@@ -7091,12 +7088,12 @@
         <v>0</v>
       </c>
       <c r="I31" s="0" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="B32" s="0" t="s">
         <v>409</v>
@@ -7117,19 +7114,19 @@
         <v>0</v>
       </c>
       <c r="G32" s="0" t="s">
-        <v>422</v>
+        <v>410</v>
       </c>
       <c r="H32" s="0" t="n">
         <f aca="false">ROUNDUP(F32/Inputs!$B$9,0)</f>
         <v>0</v>
       </c>
       <c r="I32" s="0" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B33" s="0" t="s">
         <v>378</v>
@@ -7157,15 +7154,15 @@
         <v>0</v>
       </c>
       <c r="I33" s="0" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C34" s="0" t="n">
         <v>0</v>
@@ -7182,22 +7179,22 @@
         <v>0</v>
       </c>
       <c r="G34" s="0" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="H34" s="0" t="n">
         <f aca="false">ROUNDUP(F34,0)</f>
         <v>0</v>
       </c>
       <c r="I34" s="0" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C35" s="0" t="n">
         <v>0</v>
@@ -7214,22 +7211,22 @@
         <v>0</v>
       </c>
       <c r="G35" s="0" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="H35" s="0" t="n">
         <f aca="false">ROUNDUP(F35,0)</f>
         <v>0</v>
       </c>
       <c r="I35" s="0" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C36" s="0" t="n">
         <v>19875.32</v>
@@ -7246,14 +7243,14 @@
         <v>19875.32</v>
       </c>
       <c r="G36" s="0" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="H36" s="0" t="n">
         <f aca="false">ROUNDUP(F36,0)</f>
         <v>19876</v>
       </c>
       <c r="I36" s="0" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="J36" s="0" t="n">
         <f aca="false">Inputs!$B$20*16562.8</f>
@@ -7262,10 +7259,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C37" s="0" t="n">
         <v>4556</v>
@@ -7282,14 +7279,14 @@
         <v>4556</v>
       </c>
       <c r="G37" s="0" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="H37" s="0" t="n">
         <f aca="false">ROUNDUP(F37,0)</f>
         <v>4556</v>
       </c>
       <c r="I37" s="0" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="J37" s="0" t="n">
         <f aca="false">Inputs!$B$21*1139</f>
@@ -7298,10 +7295,10 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C38" s="0" t="n">
         <v>1051.87</v>
@@ -7318,14 +7315,14 @@
         <v>1051.87</v>
       </c>
       <c r="G38" s="0" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="H38" s="0" t="n">
         <f aca="false">ROUNDUP(F38,0)</f>
         <v>1052</v>
       </c>
       <c r="I38" s="0" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="J38" s="0" t="n">
         <f aca="false">1051.87/Inputs!$B$22</f>
@@ -7334,10 +7331,10 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C39" s="0" t="n">
         <v>0</v>
@@ -7354,14 +7351,14 @@
         <v>0</v>
       </c>
       <c r="G39" s="0" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="H39" s="0" t="n">
         <f aca="false">ROUNDUP(F39,0)</f>
         <v>0</v>
       </c>
       <c r="I39" s="0" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="J39" s="0" t="n">
         <f aca="false">0*Inputs!$B$25</f>
@@ -7370,10 +7367,10 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
+        <v>452</v>
+      </c>
+      <c r="B40" s="0" t="s">
         <v>453</v>
-      </c>
-      <c r="B40" s="0" t="s">
-        <v>454</v>
       </c>
       <c r="C40" s="0" t="n">
         <v>1192.52</v>
@@ -7390,14 +7387,14 @@
         <v>1192.52</v>
       </c>
       <c r="G40" s="0" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="H40" s="0" t="n">
         <f aca="false">ROUNDUP(F40,0)</f>
         <v>1193</v>
       </c>
       <c r="I40" s="0" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="J40" s="0" t="n">
         <f aca="false">Inputs!$B$23*16562.8</f>
@@ -7406,7 +7403,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B41" s="0" t="s">
         <v>378</v>
@@ -7433,7 +7430,7 @@
         <v>6129</v>
       </c>
       <c r="I41" s="0" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="J41" s="0" t="n">
         <f aca="false">Inputs!$B$24*16562.8</f>
@@ -7442,7 +7439,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B42" s="0" t="s">
         <v>409</v>
@@ -7470,15 +7467,15 @@
         <v>0</v>
       </c>
       <c r="I42" s="0" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C43" s="0" t="n">
         <v>0</v>
@@ -7495,14 +7492,14 @@
         <v>0</v>
       </c>
       <c r="G43" s="0" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="H43" s="0" t="n">
         <f aca="false">ROUNDUP(F43,0)</f>
         <v>0</v>
       </c>
       <c r="I43" s="0" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
   </sheetData>
@@ -7530,365 +7527,365 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>463</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>464</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>465</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
+        <v>465</v>
+      </c>
+      <c r="B2" s="0" t="s">
         <v>466</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="C2" s="0" t="s">
         <v>467</v>
-      </c>
-      <c r="C2" s="0" t="s">
-        <v>468</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
+        <v>468</v>
+      </c>
+      <c r="B3" s="0" t="s">
         <v>469</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="C3" s="0" t="s">
         <v>470</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>471</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="B4" s="0" t="s">
         <v>472</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="C4" s="0" t="s">
         <v>473</v>
-      </c>
-      <c r="C4" s="0" t="s">
-        <v>474</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
+        <v>474</v>
+      </c>
+      <c r="B5" s="0" t="s">
         <v>475</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="C5" s="0" t="s">
         <v>476</v>
-      </c>
-      <c r="C5" s="0" t="s">
-        <v>477</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
+        <v>477</v>
+      </c>
+      <c r="B6" s="0" t="s">
         <v>478</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="C6" s="0" t="s">
         <v>479</v>
-      </c>
-      <c r="C6" s="0" t="s">
-        <v>480</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
+        <v>480</v>
+      </c>
+      <c r="B7" s="0" t="s">
         <v>481</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="C7" s="0" t="s">
         <v>482</v>
-      </c>
-      <c r="C7" s="0" t="s">
-        <v>483</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
+        <v>483</v>
+      </c>
+      <c r="B8" s="0" t="s">
         <v>484</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="C8" s="0" t="s">
         <v>485</v>
-      </c>
-      <c r="C8" s="0" t="s">
-        <v>486</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
+        <v>486</v>
+      </c>
+      <c r="B9" s="0" t="s">
         <v>487</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="C9" s="0" t="s">
         <v>488</v>
-      </c>
-      <c r="C9" s="0" t="s">
-        <v>489</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
+        <v>489</v>
+      </c>
+      <c r="B10" s="0" t="s">
         <v>490</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="C10" s="0" t="s">
         <v>491</v>
-      </c>
-      <c r="C10" s="0" t="s">
-        <v>492</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
+        <v>492</v>
+      </c>
+      <c r="B11" s="0" t="s">
         <v>493</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="C11" s="0" t="s">
         <v>494</v>
-      </c>
-      <c r="C11" s="0" t="s">
-        <v>495</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
+        <v>495</v>
+      </c>
+      <c r="B12" s="0" t="s">
         <v>496</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="C12" s="0" t="s">
         <v>497</v>
-      </c>
-      <c r="C12" s="0" t="s">
-        <v>498</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
+        <v>498</v>
+      </c>
+      <c r="B13" s="0" t="s">
         <v>499</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="C13" s="0" t="s">
         <v>500</v>
-      </c>
-      <c r="C13" s="0" t="s">
-        <v>501</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
+        <v>501</v>
+      </c>
+      <c r="B14" s="0" t="s">
         <v>502</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="C14" s="0" t="s">
         <v>503</v>
-      </c>
-      <c r="C14" s="0" t="s">
-        <v>504</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
+        <v>504</v>
+      </c>
+      <c r="B15" s="0" t="s">
         <v>505</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="C15" s="0" t="s">
         <v>506</v>
-      </c>
-      <c r="C15" s="0" t="s">
-        <v>507</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
+        <v>507</v>
+      </c>
+      <c r="B16" s="0" t="s">
         <v>508</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="C16" s="0" t="s">
         <v>509</v>
-      </c>
-      <c r="C16" s="0" t="s">
-        <v>510</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
+        <v>510</v>
+      </c>
+      <c r="B17" s="0" t="s">
         <v>511</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="C17" s="0" t="s">
         <v>512</v>
-      </c>
-      <c r="C17" s="0" t="s">
-        <v>513</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
+        <v>513</v>
+      </c>
+      <c r="B18" s="0" t="s">
         <v>514</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="C18" s="0" t="s">
         <v>515</v>
-      </c>
-      <c r="C18" s="0" t="s">
-        <v>516</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
+        <v>516</v>
+      </c>
+      <c r="B19" s="0" t="s">
         <v>517</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="C19" s="0" t="s">
         <v>518</v>
-      </c>
-      <c r="C19" s="0" t="s">
-        <v>519</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
+        <v>519</v>
+      </c>
+      <c r="B20" s="0" t="s">
         <v>520</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="C20" s="0" t="s">
         <v>521</v>
-      </c>
-      <c r="C20" s="0" t="s">
-        <v>522</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
+        <v>522</v>
+      </c>
+      <c r="B21" s="0" t="s">
         <v>523</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="C21" s="0" t="s">
         <v>524</v>
-      </c>
-      <c r="C21" s="0" t="s">
-        <v>525</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
+        <v>525</v>
+      </c>
+      <c r="B22" s="0" t="s">
         <v>526</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="C22" s="0" t="s">
         <v>527</v>
-      </c>
-      <c r="C22" s="0" t="s">
-        <v>528</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
+        <v>528</v>
+      </c>
+      <c r="B23" s="0" t="s">
         <v>529</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="C23" s="0" t="s">
         <v>530</v>
-      </c>
-      <c r="C23" s="0" t="s">
-        <v>531</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
+        <v>531</v>
+      </c>
+      <c r="B24" s="0" t="s">
         <v>532</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="C24" s="0" t="s">
         <v>533</v>
-      </c>
-      <c r="C24" s="0" t="s">
-        <v>534</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
+        <v>534</v>
+      </c>
+      <c r="B25" s="0" t="s">
         <v>535</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="C25" s="0" t="s">
         <v>536</v>
-      </c>
-      <c r="C25" s="0" t="s">
-        <v>537</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
+        <v>537</v>
+      </c>
+      <c r="B26" s="0" t="s">
         <v>538</v>
       </c>
-      <c r="B26" s="0" t="s">
+      <c r="C26" s="0" t="s">
         <v>539</v>
-      </c>
-      <c r="C26" s="0" t="s">
-        <v>540</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
+        <v>540</v>
+      </c>
+      <c r="B27" s="0" t="s">
         <v>541</v>
       </c>
-      <c r="B27" s="0" t="s">
+      <c r="C27" s="0" t="s">
         <v>542</v>
-      </c>
-      <c r="C27" s="0" t="s">
-        <v>543</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
+        <v>543</v>
+      </c>
+      <c r="B28" s="0" t="s">
         <v>544</v>
       </c>
-      <c r="B28" s="0" t="s">
+      <c r="C28" s="0" t="s">
         <v>545</v>
-      </c>
-      <c r="C28" s="0" t="s">
-        <v>546</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
+        <v>546</v>
+      </c>
+      <c r="B29" s="0" t="s">
         <v>547</v>
       </c>
-      <c r="B29" s="0" t="s">
+      <c r="C29" s="0" t="s">
         <v>548</v>
-      </c>
-      <c r="C29" s="0" t="s">
-        <v>549</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
+        <v>549</v>
+      </c>
+      <c r="B30" s="0" t="s">
         <v>550</v>
       </c>
-      <c r="B30" s="0" t="s">
+      <c r="C30" s="0" t="s">
         <v>551</v>
-      </c>
-      <c r="C30" s="0" t="s">
-        <v>552</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
+        <v>552</v>
+      </c>
+      <c r="B31" s="0" t="s">
         <v>553</v>
       </c>
-      <c r="B31" s="0" t="s">
+      <c r="C31" s="0" t="s">
         <v>554</v>
-      </c>
-      <c r="C31" s="0" t="s">
-        <v>555</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
+        <v>555</v>
+      </c>
+      <c r="B32" s="0" t="s">
         <v>556</v>
       </c>
-      <c r="B32" s="0" t="s">
+      <c r="C32" s="0" t="s">
         <v>557</v>
-      </c>
-      <c r="C32" s="0" t="s">
-        <v>558</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
+        <v>558</v>
+      </c>
+      <c r="B33" s="0" t="s">
         <v>559</v>
       </c>
-      <c r="B33" s="0" t="s">
+      <c r="C33" s="0" t="s">
         <v>560</v>
-      </c>
-      <c r="C33" s="0" t="s">
-        <v>561</v>
       </c>
     </row>
   </sheetData>
@@ -7920,307 +7917,307 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
+        <v>562</v>
+      </c>
+      <c r="B2" s="0" t="s">
         <v>563</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="C2" s="0" t="s">
         <v>564</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="D2" s="0" t="s">
         <v>565</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="E2" s="0" t="s">
         <v>566</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="F2" s="0" t="s">
         <v>567</v>
-      </c>
-      <c r="F2" s="0" t="s">
-        <v>568</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
+        <v>568</v>
+      </c>
+      <c r="B3" s="0" t="s">
         <v>569</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="C3" s="0" t="s">
         <v>570</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="D3" s="0" t="s">
         <v>571</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="E3" s="0" t="s">
         <v>572</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="F3" s="0" t="s">
         <v>573</v>
-      </c>
-      <c r="F3" s="0" t="s">
-        <v>574</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
+        <v>574</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>569</v>
+      </c>
+      <c r="C4" s="0" t="s">
         <v>575</v>
       </c>
-      <c r="B4" s="0" t="s">
-        <v>570</v>
-      </c>
-      <c r="C4" s="0" t="s">
+      <c r="D4" s="0" t="s">
         <v>576</v>
       </c>
-      <c r="D4" s="0" t="s">
-        <v>577</v>
-      </c>
       <c r="E4" s="0" t="s">
+        <v>572</v>
+      </c>
+      <c r="F4" s="0" t="s">
         <v>573</v>
-      </c>
-      <c r="F4" s="0" t="s">
-        <v>574</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
+        <v>577</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>569</v>
+      </c>
+      <c r="C5" s="0" t="s">
         <v>578</v>
       </c>
-      <c r="B5" s="0" t="s">
-        <v>570</v>
-      </c>
-      <c r="C5" s="0" t="s">
+      <c r="D5" s="0" t="s">
         <v>579</v>
       </c>
-      <c r="D5" s="0" t="s">
-        <v>580</v>
-      </c>
       <c r="E5" s="0" t="s">
+        <v>572</v>
+      </c>
+      <c r="F5" s="0" t="s">
         <v>573</v>
-      </c>
-      <c r="F5" s="0" t="s">
-        <v>574</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
+        <v>580</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>569</v>
+      </c>
+      <c r="C6" s="0" t="s">
         <v>581</v>
       </c>
-      <c r="B6" s="0" t="s">
-        <v>570</v>
-      </c>
-      <c r="C6" s="0" t="s">
+      <c r="D6" s="0" t="s">
         <v>582</v>
       </c>
-      <c r="D6" s="0" t="s">
-        <v>583</v>
-      </c>
       <c r="E6" s="0" t="s">
+        <v>572</v>
+      </c>
+      <c r="F6" s="0" t="s">
         <v>573</v>
-      </c>
-      <c r="F6" s="0" t="s">
-        <v>574</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
+        <v>583</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>569</v>
+      </c>
+      <c r="C7" s="0" t="s">
         <v>584</v>
       </c>
-      <c r="B7" s="0" t="s">
-        <v>570</v>
-      </c>
-      <c r="C7" s="0" t="s">
+      <c r="D7" s="0" t="s">
         <v>585</v>
-      </c>
-      <c r="D7" s="0" t="s">
-        <v>586</v>
       </c>
       <c r="E7" s="0" t="s">
         <v>185</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
+        <v>586</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>569</v>
+      </c>
+      <c r="C8" s="0" t="s">
         <v>587</v>
       </c>
-      <c r="B8" s="0" t="s">
-        <v>570</v>
-      </c>
-      <c r="C8" s="0" t="s">
+      <c r="D8" s="0" t="s">
         <v>588</v>
       </c>
-      <c r="D8" s="0" t="s">
-        <v>589</v>
-      </c>
       <c r="E8" s="0" t="s">
+        <v>572</v>
+      </c>
+      <c r="F8" s="0" t="s">
         <v>573</v>
-      </c>
-      <c r="F8" s="0" t="s">
-        <v>574</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
+        <v>589</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>569</v>
+      </c>
+      <c r="C9" s="0" t="s">
         <v>590</v>
       </c>
-      <c r="B9" s="0" t="s">
-        <v>570</v>
-      </c>
-      <c r="C9" s="0" t="s">
+      <c r="D9" s="0" t="s">
         <v>591</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="E9" s="0" t="s">
         <v>592</v>
       </c>
-      <c r="E9" s="0" t="s">
-        <v>593</v>
-      </c>
       <c r="F9" s="0" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
+        <v>593</v>
+      </c>
+      <c r="B10" s="0" t="s">
         <v>594</v>
-      </c>
-      <c r="B10" s="0" t="s">
-        <v>595</v>
       </c>
       <c r="C10" s="0" t="n">
         <v>1</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="E10" s="0" t="s">
         <v>130</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="C11" s="0" t="n">
         <v>2</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="E11" s="0" t="s">
         <v>164</v>
       </c>
       <c r="F11" s="0" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="C12" s="0" t="n">
         <v>3</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="E12" s="0" t="s">
         <v>242</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="C13" s="0" t="n">
         <v>4</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="E13" s="0" t="s">
         <v>295</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="C14" s="0" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="0" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="E14" s="0" t="s">
         <v>355</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="C15" s="0" t="n">
         <v>6</v>
       </c>
       <c r="D15" s="0" t="s">
+        <v>605</v>
+      </c>
+      <c r="E15" s="0" t="s">
         <v>606</v>
       </c>
-      <c r="E15" s="0" t="s">
-        <v>607</v>
-      </c>
       <c r="F15" s="0" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="C16" s="0" t="n">
         <v>7</v>
       </c>
       <c r="D16" s="0" t="s">
+        <v>608</v>
+      </c>
+      <c r="E16" s="0" t="s">
         <v>609</v>
       </c>
-      <c r="E16" s="0" t="s">
-        <v>610</v>
-      </c>
       <c r="F16" s="0" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
   </sheetData>
@@ -8250,366 +8247,366 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
+        <v>610</v>
+      </c>
+      <c r="B1" s="0" t="s">
         <v>611</v>
-      </c>
-      <c r="B1" s="0" t="s">
-        <v>612</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>59</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
+        <v>613</v>
+      </c>
+      <c r="B2" s="0" t="s">
         <v>614</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="C2" s="0" t="s">
         <v>615</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="D2" s="0" t="s">
         <v>616</v>
-      </c>
-      <c r="D2" s="0" t="s">
-        <v>617</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
+        <v>617</v>
+      </c>
+      <c r="B3" s="0" t="s">
         <v>618</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="C3" s="0" t="s">
+        <v>615</v>
+      </c>
+      <c r="D3" s="0" t="s">
         <v>619</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>616</v>
-      </c>
-      <c r="D3" s="0" t="s">
-        <v>620</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
+        <v>620</v>
+      </c>
+      <c r="B4" s="0" t="s">
         <v>621</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="C4" s="0" t="s">
         <v>622</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="D4" s="0" t="s">
         <v>623</v>
-      </c>
-      <c r="D4" s="0" t="s">
-        <v>624</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
+        <v>624</v>
+      </c>
+      <c r="B5" s="0" t="s">
         <v>625</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="C5" s="0" t="s">
+        <v>615</v>
+      </c>
+      <c r="D5" s="0" t="s">
         <v>626</v>
-      </c>
-      <c r="C5" s="0" t="s">
-        <v>616</v>
-      </c>
-      <c r="D5" s="0" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
+        <v>627</v>
+      </c>
+      <c r="B6" s="0" t="s">
         <v>628</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="C6" s="0" t="s">
+        <v>462</v>
+      </c>
+      <c r="D6" s="0" t="s">
         <v>629</v>
-      </c>
-      <c r="C6" s="0" t="s">
-        <v>463</v>
-      </c>
-      <c r="D6" s="0" t="s">
-        <v>630</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
+        <v>630</v>
+      </c>
+      <c r="B7" s="0" t="s">
         <v>631</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="C7" s="0" t="s">
+        <v>615</v>
+      </c>
+      <c r="D7" s="0" t="s">
         <v>632</v>
-      </c>
-      <c r="C7" s="0" t="s">
-        <v>616</v>
-      </c>
-      <c r="D7" s="0" t="s">
-        <v>633</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
+        <v>633</v>
+      </c>
+      <c r="B8" s="0" t="s">
         <v>634</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="C8" s="0" t="s">
+        <v>615</v>
+      </c>
+      <c r="D8" s="0" t="s">
         <v>635</v>
-      </c>
-      <c r="C8" s="0" t="s">
-        <v>616</v>
-      </c>
-      <c r="D8" s="0" t="s">
-        <v>636</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
+        <v>636</v>
+      </c>
+      <c r="B9" s="0" t="s">
         <v>637</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="C9" s="0" t="s">
+        <v>462</v>
+      </c>
+      <c r="D9" s="0" t="s">
         <v>638</v>
-      </c>
-      <c r="C9" s="0" t="s">
-        <v>463</v>
-      </c>
-      <c r="D9" s="0" t="s">
-        <v>639</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
+        <v>639</v>
+      </c>
+      <c r="B10" s="0" t="s">
         <v>640</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="C10" s="0" t="s">
+        <v>615</v>
+      </c>
+      <c r="D10" s="0" t="s">
         <v>641</v>
-      </c>
-      <c r="C10" s="0" t="s">
-        <v>616</v>
-      </c>
-      <c r="D10" s="0" t="s">
-        <v>642</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
+        <v>642</v>
+      </c>
+      <c r="B11" s="0" t="s">
         <v>643</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="C11" s="0" t="s">
+        <v>615</v>
+      </c>
+      <c r="D11" s="0" t="s">
         <v>644</v>
-      </c>
-      <c r="C11" s="0" t="s">
-        <v>616</v>
-      </c>
-      <c r="D11" s="0" t="s">
-        <v>645</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
+        <v>645</v>
+      </c>
+      <c r="B12" s="0" t="s">
         <v>646</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="C12" s="0" t="s">
+        <v>615</v>
+      </c>
+      <c r="D12" s="0" t="s">
         <v>647</v>
-      </c>
-      <c r="C12" s="0" t="s">
-        <v>616</v>
-      </c>
-      <c r="D12" s="0" t="s">
-        <v>648</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
+        <v>648</v>
+      </c>
+      <c r="B13" s="0" t="s">
         <v>649</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="C13" s="0" t="s">
+        <v>615</v>
+      </c>
+      <c r="D13" s="0" t="s">
         <v>650</v>
-      </c>
-      <c r="C13" s="0" t="s">
-        <v>616</v>
-      </c>
-      <c r="D13" s="0" t="s">
-        <v>651</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
+        <v>651</v>
+      </c>
+      <c r="B14" s="0" t="s">
         <v>652</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="C14" s="0" t="s">
+        <v>615</v>
+      </c>
+      <c r="D14" s="0" t="s">
         <v>653</v>
-      </c>
-      <c r="C14" s="0" t="s">
-        <v>616</v>
-      </c>
-      <c r="D14" s="0" t="s">
-        <v>654</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
+        <v>654</v>
+      </c>
+      <c r="B15" s="0" t="s">
         <v>655</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="C15" s="0" t="s">
+        <v>622</v>
+      </c>
+      <c r="D15" s="0" t="s">
         <v>656</v>
-      </c>
-      <c r="C15" s="0" t="s">
-        <v>623</v>
-      </c>
-      <c r="D15" s="0" t="s">
-        <v>657</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
+        <v>657</v>
+      </c>
+      <c r="B16" s="0" t="s">
         <v>658</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="C16" s="0" t="s">
+        <v>615</v>
+      </c>
+      <c r="D16" s="0" t="s">
         <v>659</v>
-      </c>
-      <c r="C16" s="0" t="s">
-        <v>616</v>
-      </c>
-      <c r="D16" s="0" t="s">
-        <v>660</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
+        <v>660</v>
+      </c>
+      <c r="B17" s="0" t="s">
         <v>661</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="C17" s="0" t="s">
+        <v>462</v>
+      </c>
+      <c r="D17" s="0" t="s">
         <v>662</v>
-      </c>
-      <c r="C17" s="0" t="s">
-        <v>463</v>
-      </c>
-      <c r="D17" s="0" t="s">
-        <v>663</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
+        <v>663</v>
+      </c>
+      <c r="B18" s="0" t="s">
         <v>664</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="C18" s="0" t="s">
+        <v>462</v>
+      </c>
+      <c r="D18" s="0" t="s">
         <v>665</v>
-      </c>
-      <c r="C18" s="0" t="s">
-        <v>463</v>
-      </c>
-      <c r="D18" s="0" t="s">
-        <v>666</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
+        <v>666</v>
+      </c>
+      <c r="B19" s="0" t="s">
         <v>667</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="C19" s="0" t="s">
+        <v>615</v>
+      </c>
+      <c r="D19" s="0" t="s">
         <v>668</v>
-      </c>
-      <c r="C19" s="0" t="s">
-        <v>616</v>
-      </c>
-      <c r="D19" s="0" t="s">
-        <v>669</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
+        <v>669</v>
+      </c>
+      <c r="B20" s="0" t="s">
         <v>670</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="C20" s="0" t="s">
+        <v>622</v>
+      </c>
+      <c r="D20" s="0" t="s">
         <v>671</v>
-      </c>
-      <c r="C20" s="0" t="s">
-        <v>623</v>
-      </c>
-      <c r="D20" s="0" t="s">
-        <v>672</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
+        <v>672</v>
+      </c>
+      <c r="B21" s="0" t="s">
         <v>673</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="C21" s="0" t="s">
+        <v>615</v>
+      </c>
+      <c r="D21" s="0" t="s">
         <v>674</v>
-      </c>
-      <c r="C21" s="0" t="s">
-        <v>616</v>
-      </c>
-      <c r="D21" s="0" t="s">
-        <v>675</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
+        <v>675</v>
+      </c>
+      <c r="B22" s="0" t="s">
         <v>676</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="C22" s="0" t="s">
+        <v>622</v>
+      </c>
+      <c r="D22" s="0" t="s">
         <v>677</v>
-      </c>
-      <c r="C22" s="0" t="s">
-        <v>623</v>
-      </c>
-      <c r="D22" s="0" t="s">
-        <v>678</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
+        <v>678</v>
+      </c>
+      <c r="B23" s="0" t="s">
         <v>679</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="C23" s="0" t="s">
+        <v>622</v>
+      </c>
+      <c r="D23" s="0" t="s">
         <v>680</v>
-      </c>
-      <c r="C23" s="0" t="s">
-        <v>623</v>
-      </c>
-      <c r="D23" s="0" t="s">
-        <v>681</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
+        <v>681</v>
+      </c>
+      <c r="B24" s="0" t="s">
         <v>682</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="C24" s="0" t="s">
+        <v>622</v>
+      </c>
+      <c r="D24" s="0" t="s">
         <v>683</v>
-      </c>
-      <c r="C24" s="0" t="s">
-        <v>623</v>
-      </c>
-      <c r="D24" s="0" t="s">
-        <v>684</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
+        <v>684</v>
+      </c>
+      <c r="B25" s="0" t="s">
         <v>685</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="C25" s="0" t="s">
+        <v>622</v>
+      </c>
+      <c r="D25" s="0" t="s">
         <v>686</v>
-      </c>
-      <c r="C25" s="0" t="s">
-        <v>623</v>
-      </c>
-      <c r="D25" s="0" t="s">
-        <v>687</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
+        <v>687</v>
+      </c>
+      <c r="B26" s="0" t="s">
         <v>688</v>
       </c>
-      <c r="B26" s="0" t="s">
+      <c r="C26" s="0" t="s">
+        <v>622</v>
+      </c>
+      <c r="D26" s="0" t="s">
         <v>689</v>
-      </c>
-      <c r="C26" s="0" t="s">
-        <v>623</v>
-      </c>
-      <c r="D26" s="0" t="s">
-        <v>690</v>
       </c>
     </row>
   </sheetData>
@@ -8633,12 +8630,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
   </sheetData>

</xml_diff>